<commit_message>
Add graph for barriers timing
</commit_message>
<xml_diff>
--- a/Data/Barriers_Timings.xlsx
+++ b/Data/Barriers_Timings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdagostino\Desktop\GITHUB\TRoot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950C4F5D-BF01-4A01-A50D-1E754E069440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76CF6192-C21D-4795-A0C8-284FF2828589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63B9FBB3-06A1-4971-A271-7E09DE33913A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63B9FBB3-06A1-4971-A271-7E09DE33913A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="32">
   <si>
     <t>CS_id</t>
   </si>
@@ -59,9 +59,6 @@
     <t>CS</t>
   </si>
   <si>
-    <t>LC</t>
-  </si>
-  <si>
     <t>P02_F_FY_C01_Z10_01</t>
   </si>
   <si>
@@ -77,12 +74,6 @@
     <t>P04_C_FY_C01_Z10_01</t>
   </si>
   <si>
-    <t>Sub_patchy</t>
-  </si>
-  <si>
-    <t>Sub_full</t>
-  </si>
-  <si>
     <t>P04_D_BH_C01_Z20_04</t>
   </si>
   <si>
@@ -93,6 +84,54 @@
   </si>
   <si>
     <t>age</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>En.CS-Ex.LC</t>
+  </si>
+  <si>
+    <t>En.CS-Ex.Sub</t>
+  </si>
+  <si>
+    <t>Staining</t>
+  </si>
+  <si>
+    <t>BH</t>
+  </si>
+  <si>
+    <t>FY</t>
+  </si>
+  <si>
+    <t>Suberin (complete)</t>
+  </si>
+  <si>
+    <t>Lignin Cap</t>
+  </si>
+  <si>
+    <t>Suberin (patchy)</t>
+  </si>
+  <si>
+    <t>P04_A_FY_C01_Z20_04</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>Lignin</t>
+  </si>
+  <si>
+    <t>Suberin</t>
+  </si>
+  <si>
+    <t>Polarized Cap</t>
+  </si>
+  <si>
+    <t>Complete deposition</t>
+  </si>
+  <si>
+    <t>Patchy depostition</t>
   </si>
 </sst>
 </file>
@@ -464,13 +503,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3C544C0-1314-473F-9B58-F2F36F13B627}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -481,10 +524,22 @@
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -492,13 +547,22 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2">
         <v>1.58</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -506,13 +570,22 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3">
         <v>4.7300000000000004</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -520,107 +593,226 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4">
+        <v>0.93</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="D4">
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5">
+        <v>16.68</v>
+      </c>
+      <c r="G5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6">
+        <v>19.760000000000002</v>
+      </c>
+      <c r="G6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7">
         <v>0.93</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8">
+        <v>2.78</v>
+      </c>
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9">
+        <v>4.63</v>
+      </c>
+      <c r="G9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10">
+        <v>7.41</v>
+      </c>
+      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11">
+        <v>7.41</v>
+      </c>
+      <c r="G11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>14</v>
       </c>
-      <c r="D5">
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12">
         <v>16.68</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6">
-        <v>19.760000000000002</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7">
+      <c r="G12" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13">
         <v>0.93</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8">
-        <v>2.78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9">
-        <v>4.63</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10">
-        <v>7.41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11">
-        <v>7.41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="G13" t="s">
         <v>17</v>
       </c>
-      <c r="C12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12">
-        <v>16.68</v>
+      <c r="H13" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>